<commit_message>
Updates from 25/02/26 meeting
</commit_message>
<xml_diff>
--- a/Project Org/Planning/PEP Team Assigments.xlsx
+++ b/Project Org/Planning/PEP Team Assigments.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Calvi\Documents\GitHub\PerytonElectricPropulsion\Project Plan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Calvi\Documents\GitHub\PerytonElectricPropulsion\Project Org\Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD433CB1-DBE6-4212-B5FA-C09EEB67AA70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C86FFAE9-C93D-499A-9109-1157D45802D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="27">
   <si>
     <t xml:space="preserve">TEAM </t>
   </si>
@@ -75,9 +75,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t xml:space="preserve">b   </t>
-  </si>
-  <si>
     <t xml:space="preserve">Nevzat Ozbilenler </t>
   </si>
   <si>
@@ -100,6 +97,15 @@
   </si>
   <si>
     <t>Geometry and design</t>
+  </si>
+  <si>
+    <t>Ed Armstrong</t>
+  </si>
+  <si>
+    <t>Freddie Walker</t>
+  </si>
+  <si>
+    <t>Ollie Barnes</t>
   </si>
 </sst>
 </file>
@@ -491,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
@@ -499,7 +505,7 @@
     <col min="3" max="3" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -510,14 +516,14 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
         <v>2</v>
@@ -526,7 +532,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A4" s="2"/>
       <c r="B4" s="3" t="s">
         <v>3</v>
@@ -535,21 +541,21 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="2"/>
       <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="8"/>
     </row>
-    <row r="7" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A7" s="2"/>
       <c r="B7" s="3" t="s">
         <v>6</v>
@@ -558,83 +564,80 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A8" s="2"/>
       <c r="B8" s="5" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="4"/>
     </row>
-    <row r="9" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="2"/>
       <c r="B9" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A10" s="2"/>
       <c r="B10" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G10" t="s">
         <v>15</v>
       </c>
-      <c r="H10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A11" s="2"/>
       <c r="B11" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="2"/>
       <c r="B12" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A13" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="8"/>
     </row>
-    <row r="14" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2"/>
       <c r="B14" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C14" s="4"/>
     </row>
-    <row r="15" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="2"/>
       <c r="B15" s="5" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="4"/>
     </row>
-    <row r="16" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="2"/>
       <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="18" x14ac:dyDescent="0.35">
@@ -686,21 +689,27 @@
       <c r="B23" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="4"/>
+      <c r="C23" s="4" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="24" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A24" s="2"/>
       <c r="B24" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C24" s="4"/>
+      <c r="C24" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="25" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A25" s="2"/>
       <c r="B25" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C25" s="4"/>
+      <c r="C25" s="4" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="26" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A26" s="2"/>

</xml_diff>